<commit_message>
Todo acerca de linealidad y csv
</commit_message>
<xml_diff>
--- a/Exp5b_Malus_camara/malus_mean_area1.xlsx
+++ b/Exp5b_Malus_camara/malus_mean_area1.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unaledu-my.sharepoint.com/personal/apinzonh_unal_edu_co/Documents/Docs/Universidad/2024-2/Mediciones en Óptica/2024-II_Mediciones_Opticas/Exp5b_Malus_camara/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="59" documentId="8_{3E6BDB94-D64E-49CF-91D2-08F85EE221FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F10C9B38-7804-4079-835B-3AAA0A86EEA9}"/>
+  <xr:revisionPtr revIDLastSave="55" documentId="8_{3E6BDB94-D64E-49CF-91D2-08F85EE221FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABD83D9E-EB88-406A-926D-13E8AF9E6EAA}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{D4BC4EA5-8AE6-4159-9643-BD6D92E7A69E}"/>
   </bookViews>
   <sheets>
     <sheet name="info" sheetId="4" r:id="rId1"/>
     <sheet name="red" sheetId="1" r:id="rId2"/>
-    <sheet name="blue" sheetId="2" r:id="rId3"/>
-    <sheet name="green" sheetId="3" r:id="rId4"/>
+    <sheet name="green" sheetId="3" r:id="rId3"/>
+    <sheet name="blue" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -62,23 +62,15 @@
     <t>degree</t>
   </si>
   <si>
-    <t>circle with parameters: x=1224, y=720, w=1794, h=1761</t>
+    <t>This data is for an oval area about: x = 1710, y=1368, w=576, h=558</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -106,9 +98,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -840,10 +831,10 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>189.64500000000001</v>
+        <v>251.92699999999999</v>
       </c>
       <c r="C2">
-        <v>43.2836</v>
+        <v>7.1338999999999997</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -854,10 +845,10 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>188.893</v>
+        <v>251.57900000000001</v>
       </c>
       <c r="C3">
-        <v>43.310299999999998</v>
+        <v>7.5762</v>
       </c>
       <c r="D3">
         <v>5</v>
@@ -868,10 +859,10 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>187.62100000000001</v>
+        <v>250.98400000000001</v>
       </c>
       <c r="C4">
-        <v>43.307099999999998</v>
+        <v>8.1880000000000006</v>
       </c>
       <c r="D4">
         <v>10</v>
@@ -882,10 +873,10 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>185.024</v>
+        <v>249.61500000000001</v>
       </c>
       <c r="C5">
-        <v>43.232700000000001</v>
+        <v>9.5024999999999995</v>
       </c>
       <c r="D5">
         <v>5</v>
@@ -896,10 +887,10 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>181.01400000000001</v>
+        <v>247.042</v>
       </c>
       <c r="C6">
-        <v>43.071399999999997</v>
+        <v>11.4838</v>
       </c>
       <c r="D6">
         <v>20</v>
@@ -910,10 +901,10 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>175.667</v>
+        <v>242.61699999999999</v>
       </c>
       <c r="C7">
-        <v>42.590400000000002</v>
+        <v>13.8599</v>
       </c>
       <c r="D7">
         <v>25</v>
@@ -924,10 +915,10 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>169.29300000000001</v>
+        <v>236.17</v>
       </c>
       <c r="C8">
-        <v>41.8215</v>
+        <v>16.162800000000001</v>
       </c>
       <c r="D8">
         <v>30</v>
@@ -938,10 +929,10 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>160.66399999999999</v>
+        <v>225.97499999999999</v>
       </c>
       <c r="C9">
-        <v>40.423999999999999</v>
+        <v>17.914000000000001</v>
       </c>
       <c r="D9">
         <v>35</v>
@@ -952,10 +943,10 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>151.285</v>
+        <v>213.797</v>
       </c>
       <c r="C10">
-        <v>38.591700000000003</v>
+        <v>18.187000000000001</v>
       </c>
       <c r="D10">
         <v>40</v>
@@ -966,10 +957,10 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>140.238</v>
+        <v>198.977</v>
       </c>
       <c r="C11">
-        <v>36.300199999999997</v>
+        <v>17.615600000000001</v>
       </c>
       <c r="D11">
         <v>45</v>
@@ -980,10 +971,10 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>120.926</v>
+        <v>173.30099999999999</v>
       </c>
       <c r="C12">
-        <v>32.3523</v>
+        <v>15.3246</v>
       </c>
       <c r="D12">
         <v>55</v>
@@ -994,10 +985,10 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>98.277000000000001</v>
+        <v>142.79599999999999</v>
       </c>
       <c r="C13">
-        <v>27.5503</v>
+        <v>13.610300000000001</v>
       </c>
       <c r="D13">
         <v>60</v>
@@ -1008,10 +999,10 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>80.111999999999995</v>
+        <v>118.283</v>
       </c>
       <c r="C14">
-        <v>23.669</v>
+        <v>11.9643</v>
       </c>
       <c r="D14">
         <v>65</v>
@@ -1022,10 +1013,10 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>64.72</v>
+        <v>97.451999999999998</v>
       </c>
       <c r="C15">
-        <v>20.201599999999999</v>
+        <v>10.2807</v>
       </c>
       <c r="D15">
         <v>70</v>
@@ -1036,10 +1027,10 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>25.986999999999998</v>
+        <v>43.530999999999999</v>
       </c>
       <c r="C16">
-        <v>11.0344</v>
+        <v>6.0610999999999997</v>
       </c>
       <c r="D16">
         <v>80</v>
@@ -1050,10 +1041,10 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>1.133</v>
+        <v>1.5589999999999999</v>
       </c>
       <c r="C17">
-        <v>1.5585</v>
+        <v>1.7463</v>
       </c>
       <c r="D17">
         <v>90</v>
@@ -1064,10 +1055,10 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>15.935</v>
+        <v>28.602</v>
       </c>
       <c r="C18">
-        <v>7.8014999999999999</v>
+        <v>5.1422999999999996</v>
       </c>
       <c r="D18">
         <v>100</v>
@@ -1078,10 +1069,10 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>54.246000000000002</v>
+        <v>82.933999999999997</v>
       </c>
       <c r="C19">
-        <v>17.649999999999999</v>
+        <v>9.1209000000000007</v>
       </c>
       <c r="D19">
         <v>110</v>
@@ -1092,10 +1083,10 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>89.924999999999997</v>
+        <v>131.44300000000001</v>
       </c>
       <c r="C20">
-        <v>25.672699999999999</v>
+        <v>12.7021</v>
       </c>
       <c r="D20">
         <v>120</v>
@@ -1106,10 +1097,10 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>123.333</v>
+        <v>176.22</v>
       </c>
       <c r="C21">
-        <v>32.748100000000001</v>
+        <v>16.007899999999999</v>
       </c>
       <c r="D21">
         <v>130</v>
@@ -1120,10 +1111,10 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>145.89500000000001</v>
+        <v>206.41900000000001</v>
       </c>
       <c r="C22">
-        <v>37.429699999999997</v>
+        <v>17.869</v>
       </c>
       <c r="D22">
         <v>140</v>
@@ -1134,10 +1125,10 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>165.78299999999999</v>
+        <v>231.941</v>
       </c>
       <c r="C23">
-        <v>41.2363</v>
+        <v>16.941500000000001</v>
       </c>
       <c r="D23">
         <v>150</v>
@@ -1148,10 +1139,10 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>179.58</v>
+        <v>245.78299999999999</v>
       </c>
       <c r="C24">
-        <v>42.981400000000001</v>
+        <v>12.159000000000001</v>
       </c>
       <c r="D24">
         <v>160</v>
@@ -1162,10 +1153,10 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>186.661</v>
+        <v>250.47399999999999</v>
       </c>
       <c r="C25">
-        <v>43.341700000000003</v>
+        <v>8.6484000000000005</v>
       </c>
       <c r="D25">
         <v>170</v>
@@ -1176,10 +1167,10 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>190.399</v>
+        <v>252.08500000000001</v>
       </c>
       <c r="C26">
-        <v>43.294400000000003</v>
+        <v>6.8571</v>
       </c>
       <c r="D26">
         <v>180</v>
@@ -1190,10 +1181,10 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>188.25399999999999</v>
+        <v>251.238</v>
       </c>
       <c r="C27">
-        <v>43.3459</v>
+        <v>7.8346</v>
       </c>
       <c r="D27">
         <v>190</v>
@@ -1204,10 +1195,10 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>182.55099999999999</v>
+        <v>247.87200000000001</v>
       </c>
       <c r="C28">
-        <v>43.186700000000002</v>
+        <v>10.750999999999999</v>
       </c>
       <c r="D28">
         <v>200</v>
@@ -1218,10 +1209,10 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>170.53100000000001</v>
+        <v>237.12100000000001</v>
       </c>
       <c r="C29">
-        <v>41.950600000000001</v>
+        <v>15.633599999999999</v>
       </c>
       <c r="D29">
         <v>210</v>
@@ -1232,10 +1223,10 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>152.27000000000001</v>
+        <v>214.65299999999999</v>
       </c>
       <c r="C30">
-        <v>38.689799999999998</v>
+        <v>17.751000000000001</v>
       </c>
       <c r="D30">
         <v>220</v>
@@ -1246,10 +1237,10 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>127.577</v>
+        <v>181.63200000000001</v>
       </c>
       <c r="C31">
-        <v>33.601300000000002</v>
+        <v>15.722</v>
       </c>
       <c r="D31">
         <v>230</v>
@@ -1260,10 +1251,10 @@
         <v>31</v>
       </c>
       <c r="B32">
-        <v>98.956999999999994</v>
+        <v>143.35499999999999</v>
       </c>
       <c r="C32">
-        <v>27.6404</v>
+        <v>13.0022</v>
       </c>
       <c r="D32">
         <v>240</v>
@@ -1274,10 +1265,10 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>64.156000000000006</v>
+        <v>96.346000000000004</v>
       </c>
       <c r="C33">
-        <v>20.003499999999999</v>
+        <v>9.7401</v>
       </c>
       <c r="D33">
         <v>250</v>
@@ -1288,10 +1279,10 @@
         <v>33</v>
       </c>
       <c r="B34">
-        <v>28.786000000000001</v>
+        <v>47.274999999999999</v>
       </c>
       <c r="C34">
-        <v>11.717599999999999</v>
+        <v>6.0663</v>
       </c>
       <c r="D34">
         <v>260</v>
@@ -1302,10 +1293,10 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>1.0940000000000001</v>
+        <v>1.56</v>
       </c>
       <c r="C35">
-        <v>1.5234000000000001</v>
+        <v>1.7184999999999999</v>
       </c>
       <c r="D35">
         <v>270</v>
@@ -1316,10 +1307,10 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>15.835000000000001</v>
+        <v>28.436</v>
       </c>
       <c r="C36">
-        <v>7.7773000000000003</v>
+        <v>4.9446000000000003</v>
       </c>
       <c r="D36">
         <v>280</v>
@@ -1330,10 +1321,10 @@
         <v>36</v>
       </c>
       <c r="B37">
-        <v>54.472999999999999</v>
+        <v>83.123000000000005</v>
       </c>
       <c r="C37">
-        <v>17.695499999999999</v>
+        <v>8.7566000000000006</v>
       </c>
       <c r="D37">
         <v>290</v>
@@ -1344,10 +1335,10 @@
         <v>37</v>
       </c>
       <c r="B38">
-        <v>88.796999999999997</v>
+        <v>129.86699999999999</v>
       </c>
       <c r="C38">
-        <v>25.399899999999999</v>
+        <v>12.070499999999999</v>
       </c>
       <c r="D38">
         <v>300</v>
@@ -1358,10 +1349,10 @@
         <v>38</v>
       </c>
       <c r="B39">
-        <v>123.462</v>
+        <v>176.404</v>
       </c>
       <c r="C39">
-        <v>32.718400000000003</v>
+        <v>15.415699999999999</v>
       </c>
       <c r="D39">
         <v>310</v>
@@ -1372,10 +1363,10 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>145.238</v>
+        <v>205.53200000000001</v>
       </c>
       <c r="C40">
-        <v>37.215400000000002</v>
+        <v>17.3688</v>
       </c>
       <c r="D40">
         <v>320</v>
@@ -1386,10 +1377,10 @@
         <v>40</v>
       </c>
       <c r="B41">
-        <v>165.83</v>
+        <v>232.018</v>
       </c>
       <c r="C41">
-        <v>41.153500000000001</v>
+        <v>16.671099999999999</v>
       </c>
       <c r="D41">
         <v>330</v>
@@ -1400,10 +1391,10 @@
         <v>41</v>
       </c>
       <c r="B42">
-        <v>179.92500000000001</v>
+        <v>246.07</v>
       </c>
       <c r="C42">
-        <v>42.8979</v>
+        <v>11.843500000000001</v>
       </c>
       <c r="D42">
         <v>340</v>
@@ -1414,10 +1405,10 @@
         <v>42</v>
       </c>
       <c r="B43">
-        <v>186.82599999999999</v>
+        <v>250.64400000000001</v>
       </c>
       <c r="C43">
-        <v>43.200899999999997</v>
+        <v>8.3710000000000004</v>
       </c>
       <c r="D43">
         <v>350</v>
@@ -1428,10 +1419,10 @@
         <v>43</v>
       </c>
       <c r="B44">
-        <v>190.30600000000001</v>
+        <v>252.21799999999999</v>
       </c>
       <c r="C44">
-        <v>43.209400000000002</v>
+        <v>6.6296999999999997</v>
       </c>
       <c r="D44">
         <v>360</v>
@@ -1443,6 +1434,632 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE00925D-E94D-484B-8EBE-4BCDAE1CA0E0}">
+  <dimension ref="A1:D44"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>251.66399999999999</v>
+      </c>
+      <c r="C2">
+        <v>7.3623000000000003</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>251.36</v>
+      </c>
+      <c r="C3">
+        <v>7.7474999999999996</v>
+      </c>
+      <c r="D3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>250.69900000000001</v>
+      </c>
+      <c r="C4">
+        <v>8.3937000000000008</v>
+      </c>
+      <c r="D4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>249.11199999999999</v>
+      </c>
+      <c r="C5">
+        <v>9.8444000000000003</v>
+      </c>
+      <c r="D5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>246.411</v>
+      </c>
+      <c r="C6">
+        <v>11.7784</v>
+      </c>
+      <c r="D6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>241.46700000000001</v>
+      </c>
+      <c r="C7">
+        <v>14.3177</v>
+      </c>
+      <c r="D7">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>235.02</v>
+      </c>
+      <c r="C8">
+        <v>16.4161</v>
+      </c>
+      <c r="D8">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>225.00200000000001</v>
+      </c>
+      <c r="C9">
+        <v>18.052800000000001</v>
+      </c>
+      <c r="D9">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>212.99299999999999</v>
+      </c>
+      <c r="C10">
+        <v>18.3797</v>
+      </c>
+      <c r="D10">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>198.4</v>
+      </c>
+      <c r="C11">
+        <v>17.902999999999999</v>
+      </c>
+      <c r="D11">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>171.04900000000001</v>
+      </c>
+      <c r="C12">
+        <v>15.521000000000001</v>
+      </c>
+      <c r="D12">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>140.875</v>
+      </c>
+      <c r="C13">
+        <v>13.7081</v>
+      </c>
+      <c r="D13">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>116.886</v>
+      </c>
+      <c r="C14">
+        <v>12.0085</v>
+      </c>
+      <c r="D14">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>96.42</v>
+      </c>
+      <c r="C15">
+        <v>10.2753</v>
+      </c>
+      <c r="D15">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>42.82</v>
+      </c>
+      <c r="C16">
+        <v>6.0377999999999998</v>
+      </c>
+      <c r="D16">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>1.0169999999999999</v>
+      </c>
+      <c r="C17">
+        <v>0.91420000000000001</v>
+      </c>
+      <c r="D17">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <v>27.466000000000001</v>
+      </c>
+      <c r="C18">
+        <v>4.5109000000000004</v>
+      </c>
+      <c r="D18">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <v>82.239000000000004</v>
+      </c>
+      <c r="C19">
+        <v>9.1351999999999993</v>
+      </c>
+      <c r="D19">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>130.07499999999999</v>
+      </c>
+      <c r="C20">
+        <v>12.756</v>
+      </c>
+      <c r="D20">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>174.053</v>
+      </c>
+      <c r="C21">
+        <v>16.1417</v>
+      </c>
+      <c r="D21">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22">
+        <v>203.72399999999999</v>
+      </c>
+      <c r="C22">
+        <v>18.050899999999999</v>
+      </c>
+      <c r="D22">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23">
+        <v>229.97800000000001</v>
+      </c>
+      <c r="C23">
+        <v>17.347100000000001</v>
+      </c>
+      <c r="D23">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <v>244.352</v>
+      </c>
+      <c r="C24">
+        <v>12.9108</v>
+      </c>
+      <c r="D24">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <v>250.095</v>
+      </c>
+      <c r="C25">
+        <v>8.9257000000000009</v>
+      </c>
+      <c r="D25">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26">
+        <v>251.65299999999999</v>
+      </c>
+      <c r="C26">
+        <v>7.3390000000000004</v>
+      </c>
+      <c r="D26">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27">
+        <v>250.869</v>
+      </c>
+      <c r="C27">
+        <v>8.1771999999999991</v>
+      </c>
+      <c r="D27">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28">
+        <v>246.52600000000001</v>
+      </c>
+      <c r="C28">
+        <v>11.6257</v>
+      </c>
+      <c r="D28">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29">
+        <v>235.09200000000001</v>
+      </c>
+      <c r="C29">
+        <v>16.161000000000001</v>
+      </c>
+      <c r="D29">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>211.58600000000001</v>
+      </c>
+      <c r="C30">
+        <v>17.9467</v>
+      </c>
+      <c r="D30">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>180.239</v>
+      </c>
+      <c r="C31">
+        <v>16.025099999999998</v>
+      </c>
+      <c r="D31">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <v>141.44900000000001</v>
+      </c>
+      <c r="C32">
+        <v>13.123900000000001</v>
+      </c>
+      <c r="D32">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>95.366</v>
+      </c>
+      <c r="C33">
+        <v>9.7437000000000005</v>
+      </c>
+      <c r="D33">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>45.262999999999998</v>
+      </c>
+      <c r="C34">
+        <v>5.9470000000000001</v>
+      </c>
+      <c r="D34">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="C35">
+        <v>0.9304</v>
+      </c>
+      <c r="D35">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>26.805</v>
+      </c>
+      <c r="C36">
+        <v>4.2751000000000001</v>
+      </c>
+      <c r="D36">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>82.396000000000001</v>
+      </c>
+      <c r="C37">
+        <v>8.7306000000000008</v>
+      </c>
+      <c r="D37">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>128.517</v>
+      </c>
+      <c r="C38">
+        <v>12.0884</v>
+      </c>
+      <c r="D38">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>174.29599999999999</v>
+      </c>
+      <c r="C39">
+        <v>15.490500000000001</v>
+      </c>
+      <c r="D39">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>204.07599999999999</v>
+      </c>
+      <c r="C40">
+        <v>17.516100000000002</v>
+      </c>
+      <c r="D40">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>230.58699999999999</v>
+      </c>
+      <c r="C41">
+        <v>16.8674</v>
+      </c>
+      <c r="D41">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <v>244.77099999999999</v>
+      </c>
+      <c r="C42">
+        <v>12.514799999999999</v>
+      </c>
+      <c r="D42">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43">
+        <v>250.376</v>
+      </c>
+      <c r="C43">
+        <v>8.5606000000000009</v>
+      </c>
+      <c r="D43">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44">
+        <v>251.964</v>
+      </c>
+      <c r="C44">
+        <v>6.8990999999999998</v>
+      </c>
+      <c r="D44">
+        <v>360</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09E1CC90-8FF6-4129-80FB-CB9B9989C06A}">
   <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1466,10 +2083,10 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>198.137</v>
+        <v>253.08699999999999</v>
       </c>
       <c r="C2">
-        <v>39.544199999999996</v>
+        <v>5.0434999999999999</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -1480,10 +2097,10 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>198.18100000000001</v>
+        <v>252.994</v>
       </c>
       <c r="C3">
-        <v>39.491100000000003</v>
+        <v>5.1535000000000002</v>
       </c>
       <c r="D3">
         <v>5</v>
@@ -1494,10 +2111,10 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>196.02</v>
+        <v>252.392</v>
       </c>
       <c r="C4">
-        <v>39.67</v>
+        <v>5.9385000000000003</v>
       </c>
       <c r="D4">
         <v>10</v>
@@ -1508,10 +2125,10 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>193.81399999999999</v>
+        <v>251.483</v>
       </c>
       <c r="C5">
-        <v>39.697400000000002</v>
+        <v>6.9558999999999997</v>
       </c>
       <c r="D5">
         <v>5</v>
@@ -1522,10 +2139,10 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>189.55699999999999</v>
+        <v>249.26400000000001</v>
       </c>
       <c r="C6">
-        <v>39.726900000000001</v>
+        <v>8.8948999999999998</v>
       </c>
       <c r="D6">
         <v>20</v>
@@ -1536,10 +2153,10 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>183.81399999999999</v>
+        <v>245.15799999999999</v>
       </c>
       <c r="C7">
-        <v>39.459800000000001</v>
+        <v>11.344200000000001</v>
       </c>
       <c r="D7">
         <v>25</v>
@@ -1550,10 +2167,10 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>177.73400000000001</v>
+        <v>239.30600000000001</v>
       </c>
       <c r="C8">
-        <v>38.834499999999998</v>
+        <v>13.601699999999999</v>
       </c>
       <c r="D8">
         <v>30</v>
@@ -1564,10 +2181,10 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>168.68299999999999</v>
+        <v>228.935</v>
       </c>
       <c r="C9">
-        <v>37.561100000000003</v>
+        <v>15.450900000000001</v>
       </c>
       <c r="D9">
         <v>35</v>
@@ -1578,10 +2195,10 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>158.25800000000001</v>
+        <v>215.672</v>
       </c>
       <c r="C10">
-        <v>35.759500000000003</v>
+        <v>15.781000000000001</v>
       </c>
       <c r="D10">
         <v>40</v>
@@ -1592,10 +2209,10 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>146.80699999999999</v>
+        <v>200.721</v>
       </c>
       <c r="C11">
-        <v>33.622399999999999</v>
+        <v>15.166600000000001</v>
       </c>
       <c r="D11">
         <v>45</v>
@@ -1606,10 +2223,10 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>125.02200000000001</v>
+        <v>172.721</v>
       </c>
       <c r="C12">
-        <v>29.776800000000001</v>
+        <v>13.163</v>
       </c>
       <c r="D12">
         <v>55</v>
@@ -1620,10 +2237,10 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>101.755</v>
+        <v>142.32400000000001</v>
       </c>
       <c r="C13">
-        <v>25.394500000000001</v>
+        <v>11.8056</v>
       </c>
       <c r="D13">
         <v>60</v>
@@ -1634,10 +2251,10 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>83.033000000000001</v>
+        <v>117.976</v>
       </c>
       <c r="C14">
-        <v>21.917100000000001</v>
+        <v>10.4861</v>
       </c>
       <c r="D14">
         <v>65</v>
@@ -1648,10 +2265,10 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>67.132999999999996</v>
+        <v>97.141000000000005</v>
       </c>
       <c r="C15">
-        <v>18.761900000000001</v>
+        <v>9.0883000000000003</v>
       </c>
       <c r="D15">
         <v>70</v>
@@ -1662,10 +2279,10 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>26.481000000000002</v>
+        <v>42.398000000000003</v>
       </c>
       <c r="C16">
-        <v>10.1402</v>
+        <v>5.4039999999999999</v>
       </c>
       <c r="D16">
         <v>80</v>
@@ -1676,10 +2293,10 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>0.74399999999999999</v>
+        <v>1</v>
       </c>
       <c r="C17">
-        <v>1.0608</v>
+        <v>1.0984</v>
       </c>
       <c r="D17">
         <v>90</v>
@@ -1690,10 +2307,10 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>16.183</v>
+        <v>27.815999999999999</v>
       </c>
       <c r="C18">
-        <v>7.1481000000000003</v>
+        <v>4.4907000000000004</v>
       </c>
       <c r="D18">
         <v>100</v>
@@ -1704,10 +2321,10 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>56.58</v>
+        <v>83.152000000000001</v>
       </c>
       <c r="C19">
-        <v>16.469000000000001</v>
+        <v>8.1281999999999996</v>
       </c>
       <c r="D19">
         <v>110</v>
@@ -1718,10 +2335,10 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>93.501000000000005</v>
+        <v>131.51</v>
       </c>
       <c r="C20">
-        <v>23.7605</v>
+        <v>11.123200000000001</v>
       </c>
       <c r="D20">
         <v>120</v>
@@ -1732,10 +2349,10 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>127.477</v>
+        <v>175.52699999999999</v>
       </c>
       <c r="C21">
-        <v>30.065799999999999</v>
+        <v>13.7879</v>
       </c>
       <c r="D21">
         <v>130</v>
@@ -1746,10 +2363,10 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>150.50399999999999</v>
+        <v>205.55</v>
       </c>
       <c r="C22">
-        <v>34.3277</v>
+        <v>15.3461</v>
       </c>
       <c r="D22">
         <v>140</v>
@@ -1760,10 +2377,10 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>171.74799999999999</v>
+        <v>232.73500000000001</v>
       </c>
       <c r="C23">
-        <v>38.104399999999998</v>
+        <v>15.042199999999999</v>
       </c>
       <c r="D23">
         <v>150</v>
@@ -1774,10 +2391,10 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>186.09700000000001</v>
+        <v>247.048</v>
       </c>
       <c r="C24">
-        <v>39.747700000000002</v>
+        <v>10.38</v>
       </c>
       <c r="D24">
         <v>160</v>
@@ -1788,10 +2405,10 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>193.90100000000001</v>
+        <v>251.62</v>
       </c>
       <c r="C25">
-        <v>39.897300000000001</v>
+        <v>6.8052999999999999</v>
       </c>
       <c r="D25">
         <v>170</v>
@@ -1802,10 +2419,10 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>196.994</v>
+        <v>252.78800000000001</v>
       </c>
       <c r="C26">
-        <v>39.816800000000001</v>
+        <v>5.4722</v>
       </c>
       <c r="D26">
         <v>180</v>
@@ -1816,10 +2433,10 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>195.417</v>
+        <v>252.215</v>
       </c>
       <c r="C27">
-        <v>39.877699999999997</v>
+        <v>6.1773999999999996</v>
       </c>
       <c r="D27">
         <v>190</v>
@@ -1830,10 +2447,10 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>188.934</v>
+        <v>248.79300000000001</v>
       </c>
       <c r="C28">
-        <v>39.880899999999997</v>
+        <v>9.2409999999999997</v>
       </c>
       <c r="D28">
         <v>200</v>
@@ -1844,10 +2461,10 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>176.28800000000001</v>
+        <v>237.49299999999999</v>
       </c>
       <c r="C29">
-        <v>38.741300000000003</v>
+        <v>14.055099999999999</v>
       </c>
       <c r="D29">
         <v>210</v>
@@ -1858,10 +2475,10 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>157.02699999999999</v>
+        <v>213.50200000000001</v>
       </c>
       <c r="C30">
-        <v>35.494700000000002</v>
+        <v>15.4087</v>
       </c>
       <c r="D30">
         <v>220</v>
@@ -1872,10 +2489,10 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>132.05199999999999</v>
+        <v>181.02099999999999</v>
       </c>
       <c r="C31">
-        <v>30.8963</v>
+        <v>13.628399999999999</v>
       </c>
       <c r="D31">
         <v>230</v>
@@ -1886,10 +2503,10 @@
         <v>31</v>
       </c>
       <c r="B32">
-        <v>102.495</v>
+        <v>142.821</v>
       </c>
       <c r="C32">
-        <v>25.508299999999998</v>
+        <v>11.369300000000001</v>
       </c>
       <c r="D32">
         <v>240</v>
@@ -1900,10 +2517,10 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>66.569999999999993</v>
+        <v>96.007000000000005</v>
       </c>
       <c r="C33">
-        <v>18.622</v>
+        <v>8.6502999999999997</v>
       </c>
       <c r="D33">
         <v>250</v>
@@ -1914,10 +2531,10 @@
         <v>33</v>
       </c>
       <c r="B34">
-        <v>28.027999999999999</v>
+        <v>44.27</v>
       </c>
       <c r="C34">
-        <v>10.478</v>
+        <v>5.3548</v>
       </c>
       <c r="D34">
         <v>260</v>
@@ -1928,10 +2545,10 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>0.84</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="C35">
-        <v>1.1333</v>
+        <v>1.1960999999999999</v>
       </c>
       <c r="D35">
         <v>270</v>
@@ -1942,10 +2559,10 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>15.452</v>
+        <v>26.558</v>
       </c>
       <c r="C36">
-        <v>6.8766999999999996</v>
+        <v>4.2686000000000002</v>
       </c>
       <c r="D36">
         <v>280</v>
@@ -1956,10 +2573,10 @@
         <v>36</v>
       </c>
       <c r="B37">
-        <v>56.753999999999998</v>
+        <v>83.194999999999993</v>
       </c>
       <c r="C37">
-        <v>16.508700000000001</v>
+        <v>7.7423000000000002</v>
       </c>
       <c r="D37">
         <v>290</v>
@@ -1970,10 +2587,10 @@
         <v>37</v>
       </c>
       <c r="B38">
-        <v>92.637</v>
+        <v>130.36500000000001</v>
       </c>
       <c r="C38">
-        <v>23.573699999999999</v>
+        <v>10.484</v>
       </c>
       <c r="D38">
         <v>300</v>
@@ -1984,10 +2601,10 @@
         <v>38</v>
       </c>
       <c r="B39">
-        <v>127.703</v>
+        <v>175.93700000000001</v>
       </c>
       <c r="C39">
-        <v>30.090699999999998</v>
+        <v>13.164300000000001</v>
       </c>
       <c r="D39">
         <v>310</v>
@@ -1998,10 +2615,10 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>150.46</v>
+        <v>205.47399999999999</v>
       </c>
       <c r="C40">
-        <v>34.219099999999997</v>
+        <v>14.8329</v>
       </c>
       <c r="D40">
         <v>320</v>
@@ -2012,10 +2629,10 @@
         <v>40</v>
       </c>
       <c r="B41">
-        <v>172.09200000000001</v>
+        <v>233.047</v>
       </c>
       <c r="C41">
-        <v>38.030900000000003</v>
+        <v>14.6873</v>
       </c>
       <c r="D41">
         <v>330</v>
@@ -2026,10 +2643,10 @@
         <v>41</v>
       </c>
       <c r="B42">
-        <v>186.38200000000001</v>
+        <v>247.268</v>
       </c>
       <c r="C42">
-        <v>39.636299999999999</v>
+        <v>10.1051</v>
       </c>
       <c r="D42">
         <v>340</v>
@@ -2040,10 +2657,10 @@
         <v>42</v>
       </c>
       <c r="B43">
-        <v>193.99</v>
+        <v>251.77500000000001</v>
       </c>
       <c r="C43">
-        <v>39.746400000000001</v>
+        <v>6.5359999999999996</v>
       </c>
       <c r="D43">
         <v>350</v>
@@ -2054,10 +2671,10 @@
         <v>43</v>
       </c>
       <c r="B44">
-        <v>197.48099999999999</v>
+        <v>253.07599999999999</v>
       </c>
       <c r="C44">
-        <v>39.6372</v>
+        <v>4.9687000000000001</v>
       </c>
       <c r="D44">
         <v>360</v>
@@ -2066,632 +2683,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE00925D-E94D-484B-8EBE-4BCDAE1CA0E0}">
-  <dimension ref="A1:F44"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>194.87299999999999</v>
-      </c>
-      <c r="C2">
-        <v>40.456600000000002</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>194.42</v>
-      </c>
-      <c r="C3">
-        <v>40.454300000000003</v>
-      </c>
-      <c r="D3">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>192.80500000000001</v>
-      </c>
-      <c r="C4">
-        <v>40.526200000000003</v>
-      </c>
-      <c r="D4">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>189.67599999999999</v>
-      </c>
-      <c r="C5">
-        <v>40.555399999999999</v>
-      </c>
-      <c r="D5">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>185.45</v>
-      </c>
-      <c r="C6">
-        <v>40.493200000000002</v>
-      </c>
-      <c r="D6">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>179.215</v>
-      </c>
-      <c r="C7">
-        <v>40.122799999999998</v>
-      </c>
-      <c r="D7">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8">
-        <v>172.708</v>
-      </c>
-      <c r="C8">
-        <v>39.413800000000002</v>
-      </c>
-      <c r="D8">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9">
-        <v>163.98400000000001</v>
-      </c>
-      <c r="C9">
-        <v>38.146799999999999</v>
-      </c>
-      <c r="D9">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10">
-        <v>154.41</v>
-      </c>
-      <c r="C10">
-        <v>36.444200000000002</v>
-      </c>
-      <c r="D10">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11">
-        <v>143.24600000000001</v>
-      </c>
-      <c r="C11">
-        <v>34.281300000000002</v>
-      </c>
-      <c r="D11">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12">
-        <v>122.369</v>
-      </c>
-      <c r="C12">
-        <v>30.262899999999998</v>
-      </c>
-      <c r="D12">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13">
-        <v>99.644999999999996</v>
-      </c>
-      <c r="C13">
-        <v>25.753499999999999</v>
-      </c>
-      <c r="D13">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14">
-        <v>81.432000000000002</v>
-      </c>
-      <c r="C14">
-        <v>22.202200000000001</v>
-      </c>
-      <c r="D14">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15">
-        <v>65.873999999999995</v>
-      </c>
-      <c r="C15">
-        <v>19.114699999999999</v>
-      </c>
-      <c r="D15">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16">
-        <v>26.225999999999999</v>
-      </c>
-      <c r="C16">
-        <v>10.256</v>
-      </c>
-      <c r="D16">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17">
-        <v>0.70299999999999996</v>
-      </c>
-      <c r="C17">
-        <v>0.80369999999999997</v>
-      </c>
-      <c r="D17">
-        <v>90</v>
-      </c>
-      <c r="F17" s="1"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18">
-        <v>15.827</v>
-      </c>
-      <c r="C18">
-        <v>6.9490999999999996</v>
-      </c>
-      <c r="D18">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19">
-        <v>18</v>
-      </c>
-      <c r="B19">
-        <v>55.219000000000001</v>
-      </c>
-      <c r="C19">
-        <v>16.821100000000001</v>
-      </c>
-      <c r="D19">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="B20">
-        <v>91.545000000000002</v>
-      </c>
-      <c r="C20">
-        <v>24.0518</v>
-      </c>
-      <c r="D20">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21">
-        <v>124.98399999999999</v>
-      </c>
-      <c r="C21">
-        <v>30.629300000000001</v>
-      </c>
-      <c r="D21">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22">
-        <v>147.46600000000001</v>
-      </c>
-      <c r="C22">
-        <v>35.048099999999998</v>
-      </c>
-      <c r="D22">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="B23">
-        <v>168.31800000000001</v>
-      </c>
-      <c r="C23">
-        <v>38.798400000000001</v>
-      </c>
-      <c r="D23">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24">
-        <v>23</v>
-      </c>
-      <c r="B24">
-        <v>182.636</v>
-      </c>
-      <c r="C24">
-        <v>40.451999999999998</v>
-      </c>
-      <c r="D24">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25">
-        <v>24</v>
-      </c>
-      <c r="B25">
-        <v>191.41900000000001</v>
-      </c>
-      <c r="C25">
-        <v>40.6648</v>
-      </c>
-      <c r="D25">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="B26">
-        <v>194.851</v>
-      </c>
-      <c r="C26">
-        <v>40.580100000000002</v>
-      </c>
-      <c r="D26">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27">
-        <v>26</v>
-      </c>
-      <c r="B27">
-        <v>192.99</v>
-      </c>
-      <c r="C27">
-        <v>40.653700000000001</v>
-      </c>
-      <c r="D27">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28">
-        <v>27</v>
-      </c>
-      <c r="B28">
-        <v>185.56899999999999</v>
-      </c>
-      <c r="C28">
-        <v>40.632199999999997</v>
-      </c>
-      <c r="D28">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29">
-        <v>28</v>
-      </c>
-      <c r="B29">
-        <v>173.012</v>
-      </c>
-      <c r="C29">
-        <v>39.4833</v>
-      </c>
-      <c r="D29">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30">
-        <v>29</v>
-      </c>
-      <c r="B30">
-        <v>153.666</v>
-      </c>
-      <c r="C30">
-        <v>36.251899999999999</v>
-      </c>
-      <c r="D30">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31">
-        <v>30</v>
-      </c>
-      <c r="B31">
-        <v>129.79900000000001</v>
-      </c>
-      <c r="C31">
-        <v>31.6038</v>
-      </c>
-      <c r="D31">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32">
-        <v>31</v>
-      </c>
-      <c r="B32">
-        <v>100.342</v>
-      </c>
-      <c r="C32">
-        <v>25.8447</v>
-      </c>
-      <c r="D32">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33">
-        <v>32</v>
-      </c>
-      <c r="B33">
-        <v>65.293999999999997</v>
-      </c>
-      <c r="C33">
-        <v>18.9603</v>
-      </c>
-      <c r="D33">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34">
-        <v>33</v>
-      </c>
-      <c r="B34">
-        <v>28.062999999999999</v>
-      </c>
-      <c r="C34">
-        <v>10.7111</v>
-      </c>
-      <c r="D34">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35">
-        <v>34</v>
-      </c>
-      <c r="B35">
-        <v>0.747</v>
-      </c>
-      <c r="C35">
-        <v>0.82369999999999999</v>
-      </c>
-      <c r="D35">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A36">
-        <v>35</v>
-      </c>
-      <c r="B36">
-        <v>15.452</v>
-      </c>
-      <c r="C36">
-        <v>6.7956000000000003</v>
-      </c>
-      <c r="D36">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A37">
-        <v>36</v>
-      </c>
-      <c r="B37">
-        <v>55.412999999999997</v>
-      </c>
-      <c r="C37">
-        <v>16.869299999999999</v>
-      </c>
-      <c r="D37">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A38">
-        <v>37</v>
-      </c>
-      <c r="B38">
-        <v>90.397999999999996</v>
-      </c>
-      <c r="C38">
-        <v>23.794</v>
-      </c>
-      <c r="D38">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A39">
-        <v>38</v>
-      </c>
-      <c r="B39">
-        <v>125.124</v>
-      </c>
-      <c r="C39">
-        <v>30.610199999999999</v>
-      </c>
-      <c r="D39">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A40">
-        <v>39</v>
-      </c>
-      <c r="B40">
-        <v>147.71799999999999</v>
-      </c>
-      <c r="C40">
-        <v>35.0137</v>
-      </c>
-      <c r="D40">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A41">
-        <v>40</v>
-      </c>
-      <c r="B41">
-        <v>168.785</v>
-      </c>
-      <c r="C41">
-        <v>38.778700000000001</v>
-      </c>
-      <c r="D41">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A42">
-        <v>41</v>
-      </c>
-      <c r="B42">
-        <v>182.999</v>
-      </c>
-      <c r="C42">
-        <v>40.376300000000001</v>
-      </c>
-      <c r="D42">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A43">
-        <v>42</v>
-      </c>
-      <c r="B43">
-        <v>191.59100000000001</v>
-      </c>
-      <c r="C43">
-        <v>40.540900000000001</v>
-      </c>
-      <c r="D43">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A44">
-        <v>43</v>
-      </c>
-      <c r="B44">
-        <v>195.08699999999999</v>
-      </c>
-      <c r="C44">
-        <v>40.467199999999998</v>
-      </c>
-      <c r="D44">
-        <v>360</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>